<commit_message>
Improve framework classification and reports
</commit_message>
<xml_diff>
--- a/outputs/weekly/semantic_communication_papers_2026-W20.xlsx
+++ b/outputs/weekly/semantic_communication_papers_2026-W20.xlsx
@@ -647,7 +647,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>未分类</t>
+          <t>Optimization / Resource Allocation</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -747,7 +747,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Autoencoder / DeepSC</t>
+          <t>Semantic-Aware Physical Layer</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>Autoencoder / DeepSC</t>
+          <t>Optimization / Resource Allocation</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -1147,7 +1147,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Multi-Agent</t>
+          <t>Optimization / Resource Allocation</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1247,7 +1247,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>未分类</t>
+          <t>Semantic-Aware Physical Layer</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1347,7 +1347,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>Reinforcement Learning</t>
+          <t>Semantic-Aware Physical Layer</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1447,7 +1447,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>未分类</t>
+          <t>Semantic-Aware Physical Layer</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1647,7 +1647,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>Multi-Agent</t>
+          <t>Information Theory / Semantic Coding</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">

</xml_diff>

<commit_message>
Update weekly outputs after open source scan
</commit_message>
<xml_diff>
--- a/outputs/weekly/semantic_communication_papers_2026-W20.xlsx
+++ b/outputs/weekly/semantic_communication_papers_2026-W20.xlsx
@@ -10,7 +10,7 @@
     <sheet name="papers" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'papers'!$A$1:$X$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'papers'!$A$1:$Y$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X12"/>
+  <dimension ref="A1:Y12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -440,17 +440,18 @@
     <col width="42" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="42" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
     <col width="42" customWidth="1" min="15" max="15"/>
-    <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="24" customWidth="1" min="17" max="17"/>
+    <col width="42" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
     <col width="24" customWidth="1" min="18" max="18"/>
-    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="24" customWidth="1" min="19" max="19"/>
     <col width="14" customWidth="1" min="20" max="20"/>
     <col width="14" customWidth="1" min="21" max="21"/>
     <col width="14" customWidth="1" min="22" max="22"/>
     <col width="14" customWidth="1" min="23" max="23"/>
     <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -511,65 +512,70 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>arxiv_comment</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>keywords</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>is_open_source</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>code_url</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>project_url</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>open_source_evidence</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>application_scenario</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>technical_framework</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>task_type</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>modality</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>relevance_score</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>curation_status</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>last_checked_at</t>
         </is>
@@ -625,51 +631,52 @@
           <t>Despite significant advancements in communication systems, inherent limitations persist in providing reliable data transmission for emerging applications with massive data exchanges. Semantic communication offers promising solutions by extracting and transmitting meaningful information rather than raw bit sequences. However, it faces challenges from high mobility and dynamic channel conditions in wireless environments. In this paper, we design a ground-to-air network architecture that integrates a rotary-wing unmanned aerial vehicle (UAV) and ground terminals to maximize semantic transmission efficiency while maintaining low energy consumption. This approach leverages the high mobility of the UAV for flexible deployment and the data reduction capabilities of semantic communication. Therefore, we formulate a multi-objective optimization problem to simultaneously balance the total semantic transmission rate and the UAV propulsion energy consumption by jointly optimizing the UAV hovering position, semantic encoding lengths, and resource block (RB) allocation. The problem is complex, with mixed continuous and discrete variables, which necessitates an advanced optimization method. To address these challenges, we propose a novel greedy-enhanced adaptive multi-objective cellular genetic algorithm (GEAMOCell), which utilizes an adaptive neighborhood selection mechanism to balance exploration and exploitation, and employs a crowding-guided archive feedback mechanism to maintain population diversity. The simulation results demonstrate that the proposed GEAMOCell algorithm outperforms baseline algorithms in terms of convergence, semantic transmission rate, and energy efficiency.</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
         <is>
           <t>DeepSC</t>
         </is>
       </c>
-      <c r="M2" t="b">
+      <c r="N2" t="b">
         <v>0</v>
       </c>
-      <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>not_detected</t>
-        </is>
-      </c>
+      <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr">
         <is>
+          <t>source_error:papers_with_code;source_error:pdf_link_extract</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
           <t>6G / 无线通信</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t>Optimization / Resource Allocation</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>传输</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>未标注</t>
         </is>
       </c>
-      <c r="U2" t="n">
+      <c r="V2" t="n">
         <v>13.5</v>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>curated</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr">
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr">
         <is>
           <t>2026-05-15T12:17:24.844757+00:00</t>
         </is>
@@ -725,51 +732,52 @@
           <t>Semantic communication systems for goal-oriented transmission must protect task-relevant information not only through source compression but also via physical layer mapping. Existing approaches decouple constellation design and semantic encoding, exposing critical symbols to channel errors at the same rate as irrelevant ones. Contrary to this, in this paper, a joint semantic-physical layer framework is proposed, which is composed of a vector quantized-variational autoencoder that extracts discrete latent concepts, a semantic criticality indicator (SCI) that scores each concept by task relevance, and a deep reinforcement learning agent that dynamically selects the transmission subset based on instantaneous channel conditions. At the physical layer, a learned semantic-aware M -QAM constellation assigns symbol positions according to joint co-occurrence statistics and SCI scores, departing from the uniform spacing and Gray coding of standard M -QAM which minimizes average BER without regard for semantic content. We introduce a novel semantic symbol vulnerability (SSV) metric and a semantic protection probability (SPP) to quantify the exposure of task-critical symbols to decoding errors, and prove that any Gray-coded constellation is strictly suboptimal in SCI-Weighted SSV whenever the source exhibits non-uniform semantic importance and co-occurrence statistics. Simulation results demonstrate that the proposed constellation achieves near 100% SPP across modulation orders from 4-QAM to 1024-QAM versus 50% for standard constellations at high spectral efficiency, a 21:1 compression ratio with semantic quality above 0.9, generalizing across MNIST, Fashion-MNIST, and FSDD without modification.</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
         <is>
           <t>semantic communication; semantic communications; task-oriented communication</t>
         </is>
       </c>
-      <c r="M3" t="b">
+      <c r="N3" t="b">
         <v>0</v>
       </c>
-      <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>not_detected</t>
-        </is>
-      </c>
+      <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr">
         <is>
+          <t>source_error:papers_with_code</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
           <t>任务导向通信</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="S3" t="inlineStr">
         <is>
           <t>Semantic-Aware Physical Layer</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="T3" t="inlineStr">
         <is>
           <t>传输</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>未标注</t>
         </is>
       </c>
-      <c r="U3" t="n">
+      <c r="V3" t="n">
         <v>9.5</v>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>curated</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr">
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr">
         <is>
           <t>2026-05-15T12:14:29.237416+00:00</t>
         </is>
@@ -825,51 +833,52 @@
           <t>Semantic communication (SemCom) with learned encoder-decoder architectures enables end-to-end learning of compact task-oriented representations optimized for the wireless channel, reducing channel resources needed to convey task-relevant information and improving spectrum efficiency. This paper studies semantic image transmission over block Rayleigh fading with AWGN using a multi-task semantic autoencoder that jointly reconstructs images and predicts labels from the received waveform. The latent dimension (complex channel uses per source sample) serves as a cross-layer control variable governing semantic fidelity and channel resource usage. We characterize the resulting latency-task fidelity tradeoff: larger latent representations improve inference accuracy but increase service time, channel uses, and queueing delay. Building on this insight, we develop online semantic-rate controllers that adapt the latent dimension per update under a long-term semantic error constraint. A queue-aware drift-plus-penalty policy minimizes delay subject to an average semantic error cap, while a complementary age-aware policy minimizes time-average Age of Information (AoI). By adapting the semantic rate to congestion and fidelity requirements, the proposed framework improves spectrum utilization and enables timely semantic updates with significantly lower delay and AoI than fixed-rate baselines.</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
         <is>
           <t>task-oriented communication</t>
         </is>
       </c>
-      <c r="M4" t="b">
+      <c r="N4" t="b">
         <v>0</v>
       </c>
-      <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>not_detected</t>
-        </is>
-      </c>
+      <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr">
         <is>
+          <t>source_error:papers_with_code</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
           <t>6G / 无线通信</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>Optimization / Resource Allocation</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>传输</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>Image</t>
         </is>
       </c>
-      <c r="U4" t="n">
+      <c r="V4" t="n">
         <v>8</v>
       </c>
-      <c r="V4" t="inlineStr">
+      <c r="W4" t="inlineStr">
         <is>
           <t>curated</t>
         </is>
       </c>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr">
+      <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr">
         <is>
           <t>2026-05-15T12:14:58.613259+00:00</t>
         </is>
@@ -925,51 +934,52 @@
           <t>With the rapid development of intelligent services, communication objectives are shifting from humans to multi-agent (MA) systems. This transition necessitates new communication paradigms capable of supporting real-time perception, decision-making, and collaboration among agents. Semantic communication (SeC) focuses on the efficient transmission and accurate understanding of information “meaning” and is well-suited to meet the needs of Mas, such as collaborative perception, reasoning, and decision-making. However, the transmission of semantic information is still constrained by dynamic environments and the diversity of MA tasks. To address these challenges, this work proposes a COmparative learning Joint Optimal (COJO) SeC framework. This work makes three main contributions: first, it jointly optimizes the image reconstruction and classification functions designed for multi-task semantic objectives under different channel conditions, thereby improving the overall task performance of the system; second, based on input image features, compression ratio, task requirements, and channel conditions, an enhanced further compressor is designed, which obtains a training-based mask to significantly reduce the volume of transmitted data; finally, to prevent the loss of key semantic information in multi-task scenarios under channel constraints, it designs a task-driven end-to-end semantic communication training scheme.</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
         <is>
           <t>DeepSC</t>
         </is>
       </c>
-      <c r="M5" t="b">
+      <c r="N5" t="b">
         <v>0</v>
       </c>
-      <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>not_detected</t>
-        </is>
-      </c>
+      <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr">
         <is>
+          <t>source_error:papers_with_code;source_error:pdf_link_extract</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
           <t>LLM / Agent 辅助语义通信</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="S5" t="inlineStr">
         <is>
           <t>Multi-Agent</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
+      <c r="T5" t="inlineStr">
         <is>
           <t>分类/识别</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>Image</t>
         </is>
       </c>
-      <c r="U5" t="n">
+      <c r="V5" t="n">
         <v>7.5</v>
       </c>
-      <c r="V5" t="inlineStr">
+      <c r="W5" t="inlineStr">
         <is>
           <t>curated</t>
         </is>
       </c>
-      <c r="W5" t="inlineStr"/>
-      <c r="X5" t="inlineStr">
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr">
         <is>
           <t>2026-05-15T12:17:24.844490+00:00</t>
         </is>
@@ -1025,51 +1035,52 @@
           <t>Semantic communication (SC) can achieve superior coding and transmission performance based on the knowledge contained in the semantic knowledge base (KB). However, conventional KBs consist of source KBs and channel KBs, which are often costly to obtain data and limited in data scale. Fortunately, large language models (LLMs) have recently emerged with extensive knowledge and generative capabilities. Therefore, this paper proposes an SC system with LLM-enabled knowledge base (SC-LMKB), which utilizes the generation ability of LLMs to significantly enrich the KB of SC systems. In particular, we first design an LLM-enabled generation mechanism with a prompt engineering strategy for source data generation (SDG) and a cross-attention alignment method for channel data generation (CDG). However, hallucinations from LLMs may cause semantic noise, thus degrading SC performance. To mitigate the hallucination issue, a cross-domain fusion codec (CDFC) framework with a hallucination filtering phase and a cross-domain fusion phase is then proposed for SDG. In particular, the first phase filters out new data generated by the LMKB irrelevant to the original data based on semantic similarity. Then, a cross-domain fusion phase is proposed, which fuses source data with LLM-generated data based on their semantic importance, thereby enhancing task performance. Besides, a joint training objective that combines cross-entropy loss and reconstruction loss is proposed to reduce the impact of hallucination on CDG. Experiment results on three cross-modality retrieval tasks demonstrate that the proposed SC-LMKB can achieve up to 72.6\% and 90.7\% performance gains compared to conventional SC systems and LLM-enabled SC systems, respectively.</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
         <is>
           <t>DeepSC</t>
         </is>
       </c>
-      <c r="M6" t="b">
+      <c r="N6" t="b">
         <v>0</v>
       </c>
-      <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>not_detected</t>
-        </is>
-      </c>
+      <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr">
         <is>
+          <t>source_error:papers_with_code</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
           <t>LLM / Agent 辅助语义通信</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="S6" t="inlineStr">
         <is>
           <t>Foundation Model / LLM</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
+      <c r="T6" t="inlineStr">
         <is>
           <t>生成</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>未标注</t>
         </is>
       </c>
-      <c r="U6" t="n">
+      <c r="V6" t="n">
         <v>7.5</v>
       </c>
-      <c r="V6" t="inlineStr">
+      <c r="W6" t="inlineStr">
         <is>
           <t>curated</t>
         </is>
       </c>
-      <c r="W6" t="inlineStr"/>
-      <c r="X6" t="inlineStr">
+      <c r="X6" t="inlineStr"/>
+      <c r="Y6" t="inlineStr">
         <is>
           <t>2026-05-15T12:17:24.844921+00:00</t>
         </is>
@@ -1125,51 +1136,52 @@
           <t>This letter investigates the problem of energy efficient collaborative strategy for mobile embodied artificial intelligence network (MEAN) over wireless communication. In the considered model, the agents execute the tasks through collaboration, and they can switch between two operating modes based on the signal-to-noise ratio (SNR) and global collaboration. The dual-mode comprises the base station (BS)-assisted collaborative mode, in which agents make decisions through semantic communication with BS and then collaborate on tasks, and the local computing mode, in which the agents make decisions and execute tasks independently. Due to the dynamic wireless communication and flexible collaboration strategy, we jointly consider computation energy, communication energy, and task-execution energy with specific collaborative gains into a mixed-integer nonlinear programming (MINLP) optimization problem whose goal is to minimize the total system energy consumption. To solve it, we propose a lower-complexity enumeration algorithm: first, we get the optimal closed-form solution for semantic compression ratio and transmit power by proving the strict convexity. Second, we determine the scale of collaboration and the operating mode of each agent by a greedy sorting algorithm based on individual energy-saving potentials. Simulation results show that the proposed algorithm can significantly reduce the total energy consumption compared to benchmark schemes.</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
         <is>
           <t>semantic communication; semantic communications</t>
         </is>
       </c>
-      <c r="M7" t="b">
+      <c r="N7" t="b">
         <v>0</v>
       </c>
-      <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>not_detected</t>
-        </is>
-      </c>
+      <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr">
         <is>
+          <t>source_error:papers_with_code</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
           <t>6G / 无线通信</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr">
+      <c r="S7" t="inlineStr">
         <is>
           <t>Optimization / Resource Allocation</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr">
+      <c r="T7" t="inlineStr">
         <is>
           <t>传输</t>
         </is>
       </c>
-      <c r="T7" t="inlineStr">
+      <c r="U7" t="inlineStr">
         <is>
           <t>未标注</t>
         </is>
       </c>
-      <c r="U7" t="n">
+      <c r="V7" t="n">
         <v>7</v>
       </c>
-      <c r="V7" t="inlineStr">
+      <c r="W7" t="inlineStr">
         <is>
           <t>curated</t>
         </is>
       </c>
-      <c r="W7" t="inlineStr"/>
-      <c r="X7" t="inlineStr">
+      <c r="X7" t="inlineStr"/>
+      <c r="Y7" t="inlineStr">
         <is>
           <t>2026-05-15T12:14:29.237651+00:00</t>
         </is>
@@ -1225,51 +1237,52 @@
           <t>This paper proposes a novel adaptive dual-path framework for covert semantic communication (SemCom), which integrates covert information transmission with task-oriented semantic coding. Unlike conventional covert communication methods that embed hidden messages through power-domain signal superposition, our framework embeds covert data within task-specific features via semantic-level intrinsic encoding. This new architecture introduces dual encoding paths with adaptive block selection: an Explicit path for public task execution and a Stego path that jointly encodes both public and covert information through contrastive representation alignment. A Gumbel-Softmax enabled adaptive path selection mechanism dynamically activates network blocks based on task require- ments. We formulate a multi-objective optimization framework that simultaneously ensures accurate semantic understanding and reliable covert transmission. We rigorously evaluate our framework's security against a powerful, independently trained attacker. Experimental results on the Cityscapes dataset demon- strate a state-of-the-art level of covertness: our method suppresses the attacker's detection accuracy to a near-random guessing level of 56.12%. This robust security is achieved while simultaneously maintaining superior performance on the primary semantic tasks compared to the baselines.</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
         <is>
           <t>task-oriented communication; DeepSC</t>
         </is>
       </c>
-      <c r="M8" t="b">
+      <c r="N8" t="b">
         <v>0</v>
       </c>
-      <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>not_detected</t>
-        </is>
-      </c>
+      <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr">
         <is>
+          <t>source_error:papers_with_code</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
           <t>任务导向通信</t>
         </is>
       </c>
-      <c r="R8" t="inlineStr">
+      <c r="S8" t="inlineStr">
         <is>
           <t>Semantic-Aware Physical Layer</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr">
+      <c r="T8" t="inlineStr">
         <is>
           <t>传输</t>
         </is>
       </c>
-      <c r="T8" t="inlineStr">
+      <c r="U8" t="inlineStr">
         <is>
           <t>未标注</t>
         </is>
       </c>
-      <c r="U8" t="n">
+      <c r="V8" t="n">
         <v>7</v>
       </c>
-      <c r="V8" t="inlineStr">
+      <c r="W8" t="inlineStr">
         <is>
           <t>curated</t>
         </is>
       </c>
-      <c r="W8" t="inlineStr"/>
-      <c r="X8" t="inlineStr">
+      <c r="X8" t="inlineStr"/>
+      <c r="Y8" t="inlineStr">
         <is>
           <t>2026-05-15T12:14:58.613325+00:00</t>
         </is>
@@ -1325,51 +1338,52 @@
           <t>Pinching-antennas systems (PASS) offer reconfigurable wireless channels via low-cost dielectric mediums by creating line-of-sight (LoS) communication links. Most of the existing PASS cover mechanisms of equal power pinching antennas for conventional bit-based communication, whereas flexible radiation control remains largely unexplored, particularly for heterogeneous semantic and bit users. In this paper, we investigate the performance of semantic communication (SC) using an adjustable radiation model over PASS, where the coupling strength between the dielectric waveguide and each pinching antenna is determined by the antenna-waveguide spacing. Specifically, the non-orthogonal multiple access (NOMA)-assisted heterogeneous users are served by multiple pinching antennas using spacing-controlled adjustable radiation ratios. Uunder this setting, we maximize the semantic spectral efficiency (SE) subject to the bit-user quality of service (QoS) requirement, successive interference cancellation (SIC) feasibility, and the minimum adjacent antennas spacing constraint. An alternating optimization (AO) approach optimizes users power allocation and positions of pinching antennas. Simulations demonstrate the effectiveness of the proportional power PASS model in providing higher semantic SE in different geometrical and numerical settings compared to conventional benchmark schemes.</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
         <is>
           <t>DeepSC</t>
         </is>
       </c>
-      <c r="M9" t="b">
+      <c r="N9" t="b">
         <v>0</v>
       </c>
-      <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>not_detected</t>
-        </is>
-      </c>
+      <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr">
         <is>
+          <t>source_error:papers_with_code</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
           <t>6G / 无线通信</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr">
+      <c r="S9" t="inlineStr">
         <is>
           <t>Semantic-Aware Physical Layer</t>
         </is>
       </c>
-      <c r="S9" t="inlineStr">
+      <c r="T9" t="inlineStr">
         <is>
           <t>传输</t>
         </is>
       </c>
-      <c r="T9" t="inlineStr">
+      <c r="U9" t="inlineStr">
         <is>
           <t>未标注</t>
         </is>
       </c>
-      <c r="U9" t="n">
+      <c r="V9" t="n">
         <v>7</v>
       </c>
-      <c r="V9" t="inlineStr">
+      <c r="W9" t="inlineStr">
         <is>
           <t>curated</t>
         </is>
       </c>
-      <c r="W9" t="inlineStr"/>
-      <c r="X9" t="inlineStr">
+      <c r="X9" t="inlineStr"/>
+      <c r="Y9" t="inlineStr">
         <is>
           <t>2026-05-15T12:17:24.844545+00:00</t>
         </is>
@@ -1425,51 +1439,52 @@
           <t>We investigate the performance of the pinching-antenna systems (PASS) for semantic communication (SC) in both single-waveguide and multi-waveguide scenarios, under the constraints of bit-user quality of service (QoS) and bit-to-semantic decoding order in a heterogeneous users downlink non-orthogonal multiple access (NOMA). Multiple pinching antennas in the single-waveguide scenario are at a minimum adjacent spacing required to prevent mutual coupling. An alternating optimization (AO)-based algorithm optimizes users power allocation coefficients and position of pinching antennas in the single-waveguide NOMA framework. For the multi-waveguide scenario, assuming adjacent waveguides at a sufficient lateral distance apart, the waveguides power allocation subproblem is solved using monotonic optimization and minorization-maximization (MM) approach. Specifically, a lower bound surrogate is iteratively maximized under the feasibility constraints such that a non-decreasing sequence of objective is obtained. Numerical results demonstrate that the NOMA based PASS exploiting SC offers higher semantic spectral efficiency (SE) while fulfilling the bit-user QoS requirement when compared to the considered conventional fixed antenna system. Notably, the multi-waveguide scenario becomes more beneficial for creating adjustable wireless channels in stringentconditions with higher bit-user QoS and wider coverage area requirements.</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr">
         <is>
           <t>DeepSC</t>
         </is>
       </c>
-      <c r="M10" t="b">
+      <c r="N10" t="b">
         <v>0</v>
       </c>
-      <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>not_detected</t>
-        </is>
-      </c>
+      <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr">
         <is>
+          <t>source_error:papers_with_code</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
           <t>6G / 无线通信</t>
         </is>
       </c>
-      <c r="R10" t="inlineStr">
+      <c r="S10" t="inlineStr">
         <is>
           <t>Semantic-Aware Physical Layer</t>
         </is>
       </c>
-      <c r="S10" t="inlineStr">
+      <c r="T10" t="inlineStr">
         <is>
           <t>传输</t>
         </is>
       </c>
-      <c r="T10" t="inlineStr">
+      <c r="U10" t="inlineStr">
         <is>
           <t>未标注</t>
         </is>
       </c>
-      <c r="U10" t="n">
+      <c r="V10" t="n">
         <v>7</v>
       </c>
-      <c r="V10" t="inlineStr">
+      <c r="W10" t="inlineStr">
         <is>
           <t>curated</t>
         </is>
       </c>
-      <c r="W10" t="inlineStr"/>
-      <c r="X10" t="inlineStr">
+      <c r="X10" t="inlineStr"/>
+      <c r="Y10" t="inlineStr">
         <is>
           <t>2026-05-15T12:17:24.844853+00:00</t>
         </is>
@@ -1525,51 +1540,52 @@
           <t>The rapid growth of foundation model training and large-scale AI services has driven ground data centers toward unprecedented power densities, intensifying challenges in energy supply, cooling, and spatial scalability. Space Data Centers (SDCs) have emerged as a promising paradigm for hosting energy-intensive computing infrastructures in orbit, leveraging continuous solar energy and radiative cooling advantages. However, unlike ground facilities primarily constrained by power and site availability, SDCs are fundamentally limited by communication capability. The gap between petabit-scale internal data exchange in ground data centers and the gigabit-scale capacity of ground-space links forms a critical bottleneck. This article systematically analyzes communication constraints in SDC architectures and explores semantic communication as a key enabling paradigm. By transmitting compact, task-relevant semantic representations instead of raw data, uplink pressure can be substantially reduced. The feasibility of communication-efficient orbital AI infrastructures is demonstrated through the evaluation of a multi-layer heterogeneous SDC framework consisting of relay satellites and orbital computing nodes operating under coupled energy and thermal constraints. The article further outlines open research challenges toward scalable deployment.</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr">
         <is>
           <t>semantic communication; semantic communications</t>
         </is>
       </c>
-      <c r="M11" t="b">
+      <c r="N11" t="b">
         <v>0</v>
       </c>
-      <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>not_detected</t>
-        </is>
-      </c>
+      <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr">
         <is>
+          <t>source_error:papers_with_code</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
           <t>LLM / Agent 辅助语义通信</t>
         </is>
       </c>
-      <c r="R11" t="inlineStr">
+      <c r="S11" t="inlineStr">
         <is>
           <t>Foundation Model / LLM</t>
         </is>
       </c>
-      <c r="S11" t="inlineStr">
+      <c r="T11" t="inlineStr">
         <is>
           <t>传输</t>
         </is>
       </c>
-      <c r="T11" t="inlineStr">
+      <c r="U11" t="inlineStr">
         <is>
           <t>未标注</t>
         </is>
       </c>
-      <c r="U11" t="n">
+      <c r="V11" t="n">
         <v>6.5</v>
       </c>
-      <c r="V11" t="inlineStr">
+      <c r="W11" t="inlineStr">
         <is>
           <t>curated</t>
         </is>
       </c>
-      <c r="W11" t="inlineStr"/>
-      <c r="X11" t="inlineStr">
+      <c r="X11" t="inlineStr"/>
+      <c r="Y11" t="inlineStr">
         <is>
           <t>2026-05-15T12:14:29.237809+00:00</t>
         </is>
@@ -1625,58 +1641,59 @@
           <t>Shannon's information theory deliberately excludes message semantics. This paper develops a rigorous framework for semantic communication that integrates formal proof systems with Shannon-theoretic tools. We introduce an axiomatic information model comprising Lsem-definable state sets linked by computable enabling maps, and define the semantic channel as a composition of Markov kernels whose supports respect the enabling structure. A fixed proof system induces an irredundant semantic core and a derivation-depth stratification, enabling four distortion measures of increasing semantic depth: Hamming, closure, depth, and a parameterized composite. Six families of computable semantic channel invariants are defined and their inter-relationships established, including a data processing bound, a semantic Fano bound, and an ideal-channel collapse theorem. The central quantitative result is a deductive compression gain: under closure-based fidelity, the minimum block length is determined by the irredundant core size rather than the full knowledge-base size. We instantiate the framework for heterogeneous multi-agent communication, introducing an overlap decomposition that yields necessary and sufficient conditions for closure-reliable communication. A semantic bottleneck phenomenon is identified in broadcast settings: vocabulary mismatch imposes irreducible fidelity limitations even over noiseless carriers. All results are verified on an explicit Datalog instance.</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr">
         <is>
           <t>DeepSC</t>
         </is>
       </c>
-      <c r="M12" t="b">
+      <c r="N12" t="b">
         <v>0</v>
       </c>
-      <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>not_detected</t>
-        </is>
-      </c>
+      <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr">
         <is>
+          <t>source_error:papers_with_code</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
           <t>LLM / Agent 辅助语义通信</t>
         </is>
       </c>
-      <c r="R12" t="inlineStr">
+      <c r="S12" t="inlineStr">
         <is>
           <t>Information Theory / Semantic Coding</t>
         </is>
       </c>
-      <c r="S12" t="inlineStr">
+      <c r="T12" t="inlineStr">
         <is>
           <t>传输</t>
         </is>
       </c>
-      <c r="T12" t="inlineStr">
+      <c r="U12" t="inlineStr">
         <is>
           <t>未标注</t>
         </is>
       </c>
-      <c r="U12" t="n">
+      <c r="V12" t="n">
         <v>6.5</v>
       </c>
-      <c r="V12" t="inlineStr">
+      <c r="W12" t="inlineStr">
         <is>
           <t>curated</t>
         </is>
       </c>
-      <c r="W12" t="inlineStr"/>
-      <c r="X12" t="inlineStr">
+      <c r="X12" t="inlineStr"/>
+      <c r="Y12" t="inlineStr">
         <is>
           <t>2026-05-15T12:17:24.844805+00:00</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:X12"/>
+  <autoFilter ref="A1:Y12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add open source review status fields
</commit_message>
<xml_diff>
--- a/outputs/weekly/semantic_communication_papers_2026-W20.xlsx
+++ b/outputs/weekly/semantic_communication_papers_2026-W20.xlsx
@@ -10,7 +10,7 @@
     <sheet name="papers" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'papers'!$A$1:$Y$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'papers'!$A$1:$AA$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y12"/>
+  <dimension ref="A1:AA12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -441,17 +441,19 @@
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="42" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
     <col width="42" customWidth="1" min="16" max="16"/>
-    <col width="14" customWidth="1" min="17" max="17"/>
-    <col width="24" customWidth="1" min="18" max="18"/>
-    <col width="24" customWidth="1" min="19" max="19"/>
-    <col width="14" customWidth="1" min="20" max="20"/>
-    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="42" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="24" customWidth="1" min="20" max="20"/>
+    <col width="24" customWidth="1" min="21" max="21"/>
     <col width="14" customWidth="1" min="22" max="22"/>
     <col width="14" customWidth="1" min="23" max="23"/>
     <col width="14" customWidth="1" min="24" max="24"/>
     <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="14" customWidth="1" min="26" max="26"/>
+    <col width="14" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -527,55 +529,65 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
+          <t>open_source_status</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
           <t>code_url</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>project_url</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>candidate_code_urls</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>open_source_evidence</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>application_scenario</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>technical_framework</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>task_type</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>modality</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>relevance_score</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>curation_status</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>last_checked_at</t>
         </is>
@@ -640,43 +652,49 @@
       <c r="N2" t="b">
         <v>0</v>
       </c>
-      <c r="O2" t="inlineStr"/>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>not_detected</t>
+        </is>
+      </c>
       <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr">
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr">
         <is>
           <t>source_error:papers_with_code;source_error:pdf_link_extract</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>6G / 无线通信</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>Optimization / Resource Allocation</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="V2" t="inlineStr">
         <is>
           <t>传输</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>未标注</t>
         </is>
       </c>
-      <c r="V2" t="n">
+      <c r="X2" t="n">
         <v>13.5</v>
       </c>
-      <c r="W2" t="inlineStr">
+      <c r="Y2" t="inlineStr">
         <is>
           <t>curated</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr"/>
-      <c r="Y2" t="inlineStr">
+      <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr">
         <is>
           <t>2026-05-15T12:17:24.844757+00:00</t>
         </is>
@@ -741,43 +759,49 @@
       <c r="N3" t="b">
         <v>0</v>
       </c>
-      <c r="O3" t="inlineStr"/>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>not_detected</t>
+        </is>
+      </c>
       <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr">
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr">
         <is>
           <t>source_error:papers_with_code</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="T3" t="inlineStr">
         <is>
           <t>任务导向通信</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>Semantic-Aware Physical Layer</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="V3" t="inlineStr">
         <is>
           <t>传输</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>未标注</t>
         </is>
       </c>
-      <c r="V3" t="n">
+      <c r="X3" t="n">
         <v>9.5</v>
       </c>
-      <c r="W3" t="inlineStr">
+      <c r="Y3" t="inlineStr">
         <is>
           <t>curated</t>
         </is>
       </c>
-      <c r="X3" t="inlineStr"/>
-      <c r="Y3" t="inlineStr">
+      <c r="Z3" t="inlineStr"/>
+      <c r="AA3" t="inlineStr">
         <is>
           <t>2026-05-15T12:14:29.237416+00:00</t>
         </is>
@@ -842,43 +866,49 @@
       <c r="N4" t="b">
         <v>0</v>
       </c>
-      <c r="O4" t="inlineStr"/>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>not_detected</t>
+        </is>
+      </c>
       <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr">
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr">
         <is>
           <t>source_error:papers_with_code</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>6G / 无线通信</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>Optimization / Resource Allocation</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>传输</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="W4" t="inlineStr">
         <is>
           <t>Image</t>
         </is>
       </c>
-      <c r="V4" t="n">
+      <c r="X4" t="n">
         <v>8</v>
       </c>
-      <c r="W4" t="inlineStr">
+      <c r="Y4" t="inlineStr">
         <is>
           <t>curated</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr"/>
-      <c r="Y4" t="inlineStr">
+      <c r="Z4" t="inlineStr"/>
+      <c r="AA4" t="inlineStr">
         <is>
           <t>2026-05-15T12:14:58.613259+00:00</t>
         </is>
@@ -943,43 +973,49 @@
       <c r="N5" t="b">
         <v>0</v>
       </c>
-      <c r="O5" t="inlineStr"/>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>not_detected</t>
+        </is>
+      </c>
       <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr">
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr">
         <is>
           <t>source_error:papers_with_code;source_error:pdf_link_extract</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="T5" t="inlineStr">
         <is>
           <t>LLM / Agent 辅助语义通信</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>Multi-Agent</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr">
+      <c r="V5" t="inlineStr">
         <is>
           <t>分类/识别</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
+      <c r="W5" t="inlineStr">
         <is>
           <t>Image</t>
         </is>
       </c>
-      <c r="V5" t="n">
+      <c r="X5" t="n">
         <v>7.5</v>
       </c>
-      <c r="W5" t="inlineStr">
+      <c r="Y5" t="inlineStr">
         <is>
           <t>curated</t>
         </is>
       </c>
-      <c r="X5" t="inlineStr"/>
-      <c r="Y5" t="inlineStr">
+      <c r="Z5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr">
         <is>
           <t>2026-05-15T12:17:24.844490+00:00</t>
         </is>
@@ -1044,43 +1080,49 @@
       <c r="N6" t="b">
         <v>0</v>
       </c>
-      <c r="O6" t="inlineStr"/>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>not_detected</t>
+        </is>
+      </c>
       <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr">
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr">
         <is>
           <t>source_error:papers_with_code</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="T6" t="inlineStr">
         <is>
           <t>LLM / Agent 辅助语义通信</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>Foundation Model / LLM</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr">
+      <c r="V6" t="inlineStr">
         <is>
           <t>生成</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
+      <c r="W6" t="inlineStr">
         <is>
           <t>未标注</t>
         </is>
       </c>
-      <c r="V6" t="n">
+      <c r="X6" t="n">
         <v>7.5</v>
       </c>
-      <c r="W6" t="inlineStr">
+      <c r="Y6" t="inlineStr">
         <is>
           <t>curated</t>
         </is>
       </c>
-      <c r="X6" t="inlineStr"/>
-      <c r="Y6" t="inlineStr">
+      <c r="Z6" t="inlineStr"/>
+      <c r="AA6" t="inlineStr">
         <is>
           <t>2026-05-15T12:17:24.844921+00:00</t>
         </is>
@@ -1145,43 +1187,49 @@
       <c r="N7" t="b">
         <v>0</v>
       </c>
-      <c r="O7" t="inlineStr"/>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>not_detected</t>
+        </is>
+      </c>
       <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr">
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr">
         <is>
           <t>source_error:papers_with_code</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr">
+      <c r="T7" t="inlineStr">
         <is>
           <t>6G / 无线通信</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr">
+      <c r="U7" t="inlineStr">
         <is>
           <t>Optimization / Resource Allocation</t>
         </is>
       </c>
-      <c r="T7" t="inlineStr">
+      <c r="V7" t="inlineStr">
         <is>
           <t>传输</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
+      <c r="W7" t="inlineStr">
         <is>
           <t>未标注</t>
         </is>
       </c>
-      <c r="V7" t="n">
+      <c r="X7" t="n">
         <v>7</v>
       </c>
-      <c r="W7" t="inlineStr">
+      <c r="Y7" t="inlineStr">
         <is>
           <t>curated</t>
         </is>
       </c>
-      <c r="X7" t="inlineStr"/>
-      <c r="Y7" t="inlineStr">
+      <c r="Z7" t="inlineStr"/>
+      <c r="AA7" t="inlineStr">
         <is>
           <t>2026-05-15T12:14:29.237651+00:00</t>
         </is>
@@ -1246,43 +1294,49 @@
       <c r="N8" t="b">
         <v>0</v>
       </c>
-      <c r="O8" t="inlineStr"/>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>not_detected</t>
+        </is>
+      </c>
       <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>source_error:papers_with_code</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>source_error:papers_with_code;source_error:pdf_link_extract</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
         <is>
           <t>任务导向通信</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr">
+      <c r="U8" t="inlineStr">
         <is>
           <t>Semantic-Aware Physical Layer</t>
         </is>
       </c>
-      <c r="T8" t="inlineStr">
+      <c r="V8" t="inlineStr">
         <is>
           <t>传输</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr">
+      <c r="W8" t="inlineStr">
         <is>
           <t>未标注</t>
         </is>
       </c>
-      <c r="V8" t="n">
+      <c r="X8" t="n">
         <v>7</v>
       </c>
-      <c r="W8" t="inlineStr">
+      <c r="Y8" t="inlineStr">
         <is>
           <t>curated</t>
         </is>
       </c>
-      <c r="X8" t="inlineStr"/>
-      <c r="Y8" t="inlineStr">
+      <c r="Z8" t="inlineStr"/>
+      <c r="AA8" t="inlineStr">
         <is>
           <t>2026-05-15T12:14:58.613325+00:00</t>
         </is>
@@ -1347,43 +1401,49 @@
       <c r="N9" t="b">
         <v>0</v>
       </c>
-      <c r="O9" t="inlineStr"/>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>not_detected</t>
+        </is>
+      </c>
       <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr">
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr">
         <is>
           <t>source_error:papers_with_code</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr">
+      <c r="T9" t="inlineStr">
         <is>
           <t>6G / 无线通信</t>
         </is>
       </c>
-      <c r="S9" t="inlineStr">
+      <c r="U9" t="inlineStr">
         <is>
           <t>Semantic-Aware Physical Layer</t>
         </is>
       </c>
-      <c r="T9" t="inlineStr">
+      <c r="V9" t="inlineStr">
         <is>
           <t>传输</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr">
+      <c r="W9" t="inlineStr">
         <is>
           <t>未标注</t>
         </is>
       </c>
-      <c r="V9" t="n">
+      <c r="X9" t="n">
         <v>7</v>
       </c>
-      <c r="W9" t="inlineStr">
+      <c r="Y9" t="inlineStr">
         <is>
           <t>curated</t>
         </is>
       </c>
-      <c r="X9" t="inlineStr"/>
-      <c r="Y9" t="inlineStr">
+      <c r="Z9" t="inlineStr"/>
+      <c r="AA9" t="inlineStr">
         <is>
           <t>2026-05-15T12:17:24.844545+00:00</t>
         </is>
@@ -1448,43 +1508,49 @@
       <c r="N10" t="b">
         <v>0</v>
       </c>
-      <c r="O10" t="inlineStr"/>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>not_detected</t>
+        </is>
+      </c>
       <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr">
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr">
         <is>
           <t>source_error:papers_with_code</t>
         </is>
       </c>
-      <c r="R10" t="inlineStr">
+      <c r="T10" t="inlineStr">
         <is>
           <t>6G / 无线通信</t>
         </is>
       </c>
-      <c r="S10" t="inlineStr">
+      <c r="U10" t="inlineStr">
         <is>
           <t>Semantic-Aware Physical Layer</t>
         </is>
       </c>
-      <c r="T10" t="inlineStr">
+      <c r="V10" t="inlineStr">
         <is>
           <t>传输</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr">
+      <c r="W10" t="inlineStr">
         <is>
           <t>未标注</t>
         </is>
       </c>
-      <c r="V10" t="n">
+      <c r="X10" t="n">
         <v>7</v>
       </c>
-      <c r="W10" t="inlineStr">
+      <c r="Y10" t="inlineStr">
         <is>
           <t>curated</t>
         </is>
       </c>
-      <c r="X10" t="inlineStr"/>
-      <c r="Y10" t="inlineStr">
+      <c r="Z10" t="inlineStr"/>
+      <c r="AA10" t="inlineStr">
         <is>
           <t>2026-05-15T12:17:24.844853+00:00</t>
         </is>
@@ -1549,43 +1615,49 @@
       <c r="N11" t="b">
         <v>0</v>
       </c>
-      <c r="O11" t="inlineStr"/>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>not_detected</t>
+        </is>
+      </c>
       <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr">
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr">
         <is>
           <t>source_error:papers_with_code</t>
         </is>
       </c>
-      <c r="R11" t="inlineStr">
+      <c r="T11" t="inlineStr">
         <is>
           <t>LLM / Agent 辅助语义通信</t>
         </is>
       </c>
-      <c r="S11" t="inlineStr">
+      <c r="U11" t="inlineStr">
         <is>
           <t>Foundation Model / LLM</t>
         </is>
       </c>
-      <c r="T11" t="inlineStr">
+      <c r="V11" t="inlineStr">
         <is>
           <t>传输</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr">
+      <c r="W11" t="inlineStr">
         <is>
           <t>未标注</t>
         </is>
       </c>
-      <c r="V11" t="n">
+      <c r="X11" t="n">
         <v>6.5</v>
       </c>
-      <c r="W11" t="inlineStr">
+      <c r="Y11" t="inlineStr">
         <is>
           <t>curated</t>
         </is>
       </c>
-      <c r="X11" t="inlineStr"/>
-      <c r="Y11" t="inlineStr">
+      <c r="Z11" t="inlineStr"/>
+      <c r="AA11" t="inlineStr">
         <is>
           <t>2026-05-15T12:14:29.237809+00:00</t>
         </is>
@@ -1650,50 +1722,56 @@
       <c r="N12" t="b">
         <v>0</v>
       </c>
-      <c r="O12" t="inlineStr"/>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>not_detected</t>
+        </is>
+      </c>
       <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr">
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr">
         <is>
           <t>source_error:papers_with_code</t>
         </is>
       </c>
-      <c r="R12" t="inlineStr">
+      <c r="T12" t="inlineStr">
         <is>
           <t>LLM / Agent 辅助语义通信</t>
         </is>
       </c>
-      <c r="S12" t="inlineStr">
+      <c r="U12" t="inlineStr">
         <is>
           <t>Information Theory / Semantic Coding</t>
         </is>
       </c>
-      <c r="T12" t="inlineStr">
+      <c r="V12" t="inlineStr">
         <is>
           <t>传输</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr">
+      <c r="W12" t="inlineStr">
         <is>
           <t>未标注</t>
         </is>
       </c>
-      <c r="V12" t="n">
+      <c r="X12" t="n">
         <v>6.5</v>
       </c>
-      <c r="W12" t="inlineStr">
+      <c r="Y12" t="inlineStr">
         <is>
           <t>curated</t>
         </is>
       </c>
-      <c r="X12" t="inlineStr"/>
-      <c r="Y12" t="inlineStr">
+      <c r="Z12" t="inlineStr"/>
+      <c r="AA12" t="inlineStr">
         <is>
           <t>2026-05-15T12:17:24.844805+00:00</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Y12"/>
+  <autoFilter ref="A1:AA12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Improve open source review workflow
</commit_message>
<xml_diff>
--- a/outputs/weekly/semantic_communication_papers_2026-W20.xlsx
+++ b/outputs/weekly/semantic_communication_papers_2026-W20.xlsx
@@ -444,8 +444,8 @@
     <col width="14" customWidth="1" min="15" max="15"/>
     <col width="42" customWidth="1" min="16" max="16"/>
     <col width="42" customWidth="1" min="17" max="17"/>
-    <col width="14" customWidth="1" min="18" max="18"/>
-    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="42" customWidth="1" min="18" max="18"/>
+    <col width="42" customWidth="1" min="19" max="19"/>
     <col width="24" customWidth="1" min="20" max="20"/>
     <col width="24" customWidth="1" min="21" max="21"/>
     <col width="14" customWidth="1" min="22" max="22"/>
@@ -876,7 +876,7 @@
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr">
         <is>
-          <t>source_error:papers_with_code</t>
+          <t>source_error:papers_with_code;source_error:github_search</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -1090,7 +1090,7 @@
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr">
         <is>
-          <t>source_error:papers_with_code</t>
+          <t>source_error:papers_with_code;source_error:github_search</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -1304,7 +1304,7 @@
       <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr">
         <is>
-          <t>source_error:papers_with_code;source_error:pdf_link_extract</t>
+          <t>source_error:papers_with_code;source_error:github_search</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -1518,7 +1518,7 @@
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr">
         <is>
-          <t>source_error:papers_with_code</t>
+          <t>source_error:papers_with_code;source_error:github_search</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -1732,7 +1732,7 @@
       <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr">
         <is>
-          <t>source_error:papers_with_code</t>
+          <t>source_error:papers_with_code;source_error:github_search</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">

</xml_diff>